<commit_message>
Used Standard Names for Automation records
</commit_message>
<xml_diff>
--- a/src/main/resources/KPI_Field_Values.xlsx
+++ b/src/main/resources/KPI_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2208FAD9-A7BA-4099-B1AA-B06B1A5D9DBE}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D7AB79-B751-4E86-94A7-FD7B9A0F58A7}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{BDA37FF1-763A-4534-A27A-58B72EDE21C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BDA37FF1-763A-4534-A27A-58B72EDE21C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -75,7 +75,7 @@
     <t>Economic Development</t>
   </si>
   <si>
-    <t>Automation KPI</t>
+    <t>Execution KPI for Automation</t>
   </si>
 </sst>
 </file>
@@ -428,13 +428,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{263A4B3D-DD01-4D88-9D0B-35905B1C6D43}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -456,7 +456,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -467,7 +467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -478,7 +478,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -502,19 +502,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5008D992-E627-44A6-B9F5-A658F6BB18BD}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,7 +526,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
updated kpi and strategic plan
</commit_message>
<xml_diff>
--- a/src/main/resources/KPI_Field_Values.xlsx
+++ b/src/main/resources/KPI_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CFF1B4-C66C-44EA-8531-5C3B45CEF9FF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E82F68F-0744-4AD1-957D-8A358A1DF0BC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{BDA37FF1-763A-4534-A27A-58B72EDE21C5}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" xr2:uid="{BDA37FF1-763A-4534-A27A-58B72EDE21C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -75,7 +75,7 @@
     <t>Economic Development</t>
   </si>
   <si>
-    <t>Automation Execution KPI</t>
+    <t>Automation Runtime KPI</t>
   </si>
 </sst>
 </file>
@@ -428,13 +428,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{263A4B3D-DD01-4D88-9D0B-35905B1C6D43}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -456,7 +456,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -467,7 +467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -478,7 +478,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -509,13 +509,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5008D992-E627-44A6-B9F5-A658F6BB18BD}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -526,7 +526,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>

</xml_diff>